<commit_message>
Add Ansible NetBox hardware inventory collector
</commit_message>
<xml_diff>
--- a/tools/netbox/csv-import/template/inventory-template.xlsx
+++ b/tools/netbox/csv-import/template/inventory-template.xlsx
@@ -14,9 +14,12 @@
     <sheet name="Sites" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Racks" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Devices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="VLANs" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Prefixes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="IPAddresses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Interfaces" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MACAddresses" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="InventoryItems" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="VLANs" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Prefixes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="IPAddresses" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -553,34 +556,70 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VLANs</t>
+          <t>Interfaces</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>vid, name</t>
+          <t>device, name</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Prefixes</t>
+          <t>MACAddresses</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>prefix</t>
+          <t>address, device, interface</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>InventoryItems</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>device, name</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>VLANs</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>vid, name</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Prefixes</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>prefix</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>IPAddresses</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>address</t>
         </is>
@@ -592,6 +631,220 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>device</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>part_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>serial</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>srv01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DIMM_A1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>vid</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>servers</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>prefix</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>10.0.0.0/24</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -928,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -940,6 +1193,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -988,6 +1242,11 @@
           <t>serial</t>
         </is>
       </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1029,6 +1288,7 @@
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1041,19 +1301,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>vid</t>
+          <t>device</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -1063,34 +1324,42 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>type</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>100</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>srv01</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>servers</t>
+          <t>eth0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>other</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1103,32 +1372,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>prefix</t>
+          <t>address</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>device</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>interface</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -1137,20 +1412,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10.0.0.0/24</t>
+          <t>00:11:22:33:44:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>srv01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>eth0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>